<commit_message>
Nilai kelas 1 putri
</commit_message>
<xml_diff>
--- a/Soal Komputer/Penilaian kelas 1.xlsx
+++ b/Soal Komputer/Penilaian kelas 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASATIDZ\Zen\pelajaran-komputer\Soal Komputer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2033DD55-DF91-4F7A-9C07-C19B943F2237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E07A3D-CB65-450B-972F-63ACEAFD2A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Nama</t>
   </si>
@@ -85,6 +85,30 @@
   </si>
   <si>
     <t>Column1</t>
+  </si>
+  <si>
+    <t>Aina Talita Zahron</t>
+  </si>
+  <si>
+    <t>Aisyah Nurul Hafizah</t>
+  </si>
+  <si>
+    <t>Annisa Qurrotu'aini Al Adawiyah</t>
+  </si>
+  <si>
+    <t>Bilqis</t>
+  </si>
+  <si>
+    <t>Erina Liyana Zahra</t>
+  </si>
+  <si>
+    <t>Nur Humaira Safitri</t>
+  </si>
+  <si>
+    <t>Siti Sofia Azzalea</t>
+  </si>
+  <si>
+    <t>Zhafira Aqeela Zahra</t>
   </si>
 </sst>
 </file>
@@ -125,7 +149,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -141,8 +165,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED562658-8911-42A0-BC3E-BD91EC2219CA}" name="Table1" displayName="Table1" ref="A1:L8" totalsRowShown="0">
-  <autoFilter ref="A1:L8" xr:uid="{ED562658-8911-42A0-BC3E-BD91EC2219CA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ED562658-8911-42A0-BC3E-BD91EC2219CA}" name="Table1" displayName="Table1" ref="A1:L16" totalsRowShown="0">
+  <autoFilter ref="A1:L16" xr:uid="{ED562658-8911-42A0-BC3E-BD91EC2219CA}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{C50C83D3-4B7E-45E6-AAA6-663D3DE26C97}" name="Nama"/>
     <tableColumn id="12" xr3:uid="{D67BA0BD-7943-4E4D-BABD-4EA423C0AA07}" name="Column1"/>
@@ -427,7 +451,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
@@ -538,6 +562,70 @@
         <v>60</v>
       </c>
     </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="83" orientation="landscape" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Kelas 2 putra sebagian besar
</commit_message>
<xml_diff>
--- a/Soal Komputer/Penilaian kelas 1.xlsx
+++ b/Soal Komputer/Penilaian kelas 1.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ASATIDZ\Zen\pelajaran-komputer\Soal Komputer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E07A3D-CB65-450B-972F-63ACEAFD2A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB155C9-2BEB-42AD-84BF-9F660CE5046F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="1" sheetId="1" r:id="rId1"/>
+    <sheet name="2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Table1[#All]</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">الجدول2[#All]</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="49">
   <si>
     <t>Nama</t>
   </si>
@@ -109,6 +111,72 @@
   </si>
   <si>
     <t>Zhafira Aqeela Zahra</t>
+  </si>
+  <si>
+    <t>Caveman</t>
+  </si>
+  <si>
+    <t>Gambar Trofi</t>
+  </si>
+  <si>
+    <t>Gambar Pemain Bola</t>
+  </si>
+  <si>
+    <t>Gambar Klub dan Negara</t>
+  </si>
+  <si>
+    <t>Tabel</t>
+  </si>
+  <si>
+    <t>Judul</t>
+  </si>
+  <si>
+    <t>Tombol Berlangganan</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>Link Beli Tiket</t>
+  </si>
+  <si>
+    <t>Abdullah Umar Al-Hummam</t>
+  </si>
+  <si>
+    <t>Afkar Mukayyis Al Wahidi</t>
+  </si>
+  <si>
+    <t>Ammar Azzamul Haq</t>
+  </si>
+  <si>
+    <t>Fatih Alfaizi Aufa Ramadhan</t>
+  </si>
+  <si>
+    <t>Khalid Fayyadh Al Muzzammil</t>
+  </si>
+  <si>
+    <t>Muhammad Alvin Abdurrahman</t>
+  </si>
+  <si>
+    <t>Muhammad Rizky</t>
+  </si>
+  <si>
+    <t>Muhammad Rizky Suhaili</t>
+  </si>
+  <si>
+    <t>Muhammad Sano Darussalam Ro</t>
+  </si>
+  <si>
+    <t>Muhammad Yusuf Kamil Fahlevi</t>
+  </si>
+  <si>
+    <t>Thoriq Mubarok Muttaqin</t>
+  </si>
+  <si>
+    <t>Umar Abdurrosyid Assariy</t>
+  </si>
+  <si>
+    <t>عمود1</t>
   </si>
 </sst>
 </file>
@@ -180,6 +248,27 @@
     <tableColumn id="9" xr3:uid="{AF7E3E63-4178-4DE1-A3EE-E67CBCEE8F87}" name="Tebal"/>
     <tableColumn id="10" xr3:uid="{1211F08F-F646-424E-945D-51949B401355}" name="Tab"/>
     <tableColumn id="11" xr3:uid="{232EF59F-96DF-4DE6-A3B7-6732F1CA1050}" name="Table"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{89944B79-69C5-46D2-B511-4470C93D3F87}" name="الجدول2" displayName="الجدول2" ref="A1:L13" totalsRowShown="0">
+  <autoFilter ref="A1:L13" xr:uid="{89944B79-69C5-46D2-B511-4470C93D3F87}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{B5C890C0-9B1E-4ED4-9EEF-B4772178B428}" name="Nama"/>
+    <tableColumn id="12" xr3:uid="{F10677B0-3575-40BD-A9EE-A17F6A1365A7}" name="عمود1"/>
+    <tableColumn id="2" xr3:uid="{65300E4B-5B89-4EAA-9CCC-EDB4C90A88E8}" name="Caveman"/>
+    <tableColumn id="3" xr3:uid="{43AC8CAE-E188-43F1-9329-2EDB7E43EC37}" name="Selesai"/>
+    <tableColumn id="4" xr3:uid="{B1C6552E-54D5-46E2-89B1-2E41AD569090}" name="Gambar Trofi"/>
+    <tableColumn id="5" xr3:uid="{3F73FDAE-9CB5-48DE-90F8-CB06AF806154}" name="Gambar Klub dan Negara"/>
+    <tableColumn id="6" xr3:uid="{56046533-10E8-452F-8B7A-97311FD52BAE}" name="Gambar Pemain Bola"/>
+    <tableColumn id="7" xr3:uid="{E33B6662-D385-40B9-8D0C-7CD20B62DDE7}" name="Tabel"/>
+    <tableColumn id="8" xr3:uid="{2B839F65-7172-4DB4-BE51-24278D194C5E}" name="Judul"/>
+    <tableColumn id="9" xr3:uid="{02CCB3A9-5520-4B3D-85DF-503DA7020DE8}" name="Tombol Berlangganan"/>
+    <tableColumn id="10" xr3:uid="{E9F9B4AA-DD64-4805-8D7F-D540D38F8900}" name="Footer"/>
+    <tableColumn id="11" xr3:uid="{4F2F7921-7445-4753-9EA9-57B365BD0BBE}" name="Link Beli Tiket"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -633,4 +722,160 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F281D9B-A933-4152-8B6B-FC7313F6B254}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>